<commit_message>
added all answer keys and validation logic. still need  the actual checker script
</commit_message>
<xml_diff>
--- a/benchmarks/answer-keys/Answers for Source Files.xlsx
+++ b/benchmarks/answer-keys/Answers for Source Files.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Nextcloud/Documents/Code/Code-Public/archer-ai/benchmarks/answer-keys/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99957F42-2862-9446-BF4C-0750C090E2D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFF2FA01-BE8F-334C-9B85-9037BA71F02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25620" yWindow="620" windowWidth="25620" windowHeight="27040" xr2:uid="{96F3FD9E-364F-B44D-8CBB-2BB866FED4A0}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="51200" windowHeight="27040" xr2:uid="{96F3FD9E-364F-B44D-8CBB-2BB866FED4A0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="272">
   <si>
     <t>ID</t>
   </si>
@@ -624,12 +624,402 @@
   <si>
     <t>COMPLIANT</t>
   </si>
+  <si>
+    <t>Prompt</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a Python function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>get_allowed_ips(config_text)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that returns all AllowedIPs from a WireGuard peer config as a list of strings</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a Python function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>normalize_mac(mac)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that returns the MAC address in lowercase colon-separated form, or None if invalid</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a Python function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>health(cpu_temp, fan_rpm)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that returns "ok", "warn" or "critical" per the stated rules</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a Python function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>expand_cron_minutes(field)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that returns the sorted list of minutes a cron minute field matches</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a Python function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>backups_to_keep(dates, today)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that returns which backup dates to keep: last 7 daily, 4 Sundays, 3 month-starts</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a Python function </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>is_prime(n)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> that returns True if n is prime and False otherwise</t>
+    </r>
+  </si>
+  <si>
+    <t>Write a Python-flavor regex that matches only private IPv4 addresses</t>
+  </si>
+  <si>
+    <t>Write a SQL query returning the maximum temperature per station for a given day. Return only the SQL query.</t>
+  </si>
+  <si>
+    <t>Write a SQL query returning hosts with no check in the last 24 hours. Return only the SQL query.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Write a bash one-liner that prints mountpoints at 80% use or above from this </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>df -h</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> output</t>
+    </r>
+  </si>
+  <si>
+    <t>What is the only mammal capable of true sustained flight? Answer with the common name only.</t>
+  </si>
+  <si>
+    <t>What is the chemical symbol for tungsten? Answer with only the symbol.</t>
+  </si>
+  <si>
+    <t>At what temperature are the Celsius and Fahrenheit scales equal? Answer with only the number.</t>
+  </si>
+  <si>
+    <t>What is the capital city of Australia? Answer with the city name only.</t>
+  </si>
+  <si>
+    <t>How many bones are in the adult human body? Answer with only the number.</t>
+  </si>
+  <si>
+    <t>How many bits long is an IPv6 address? Answer with only the number.</t>
+  </si>
+  <si>
+    <t>What is the USDA minimum safe internal temperature for cooked chicken, in degrees Fahrenheit? Answer with only the number.</t>
+  </si>
+  <si>
+    <t>What is the past tense of the English verb "lead"? Answer with one word.</t>
+  </si>
+  <si>
+    <t>Who wrote the novel Frankenstein? Answer with the author's surname only.</t>
+  </si>
+  <si>
+    <t>In what year did the Berlin Wall fall? Answer with only the number.</t>
+  </si>
+  <si>
+    <t>Four identical 8 TB drives are in RAID5 array. What is the total usable capacity in Terabytes? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>A subnet has CIDR /27. How many usable host addresses does it contain? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>A backup starts at 22:45 and runs for 3 hours 35 minutes. At what 24-hour time does it finish? Answer as HH:MM only.</t>
+  </si>
+  <si>
+    <t>A server is considered overloaded if CPU exceeds 85% and RAM exceeds 90%, or if load average exceeds 25. CPU=88%, RAM=91%, Load=12. Return only OVERLOADED or NORMAL.</t>
+  </si>
+  <si>
+    <t>A company has 18 switches. Each switch has 48 ports. 35 ports per switch are in use. How many ports remain available across all switches? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>A UPS supplies 900 watts for 20 minutes. How many watt-hours of energy does that represent? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>ailed login attempts occur at 12:00, 12:04, 12:08, and 12:11 from the same IP. Policy locks out an IP if 3 or more failed attempts occur within any rolling 10-minute window. Return only YES or NO indicating whether the IP is locked out.</t>
+  </si>
+  <si>
+    <t>A network reserves the first 10 IPs and last 5 IPs of a /24 subnet. How many addresses remain assignable? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>A folder contains 37 daily backups. Policy keeps every backup from the most recent 7 days and deletes the rest. How many backups are deleted? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>A web server averages 120 requests per second. Peak traffic is defined as 250% of average. How many requests per second represent peak traffic? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>Return a JSON object with keys hostname, ip, and status using the values server01, 10.0.0.5, and online. Output valid JSON only.</t>
+  </si>
+  <si>
+    <t>Describe a bicycle in exactly 12 words.</t>
+  </si>
+  <si>
+    <t>Output only the following three lines and nothing else: NAME=Alice ROLE=Admin STATUS=Active</t>
+  </si>
+  <si>
+    <t>Output only the following CSV row, with no header row, no quotes, and nothing else: Chicago,Illinois,2700000</t>
+  </si>
+  <si>
+    <t>Output the word Linux in uppercase only.</t>
+  </si>
+  <si>
+    <t>Output exactly 20 X characters and nothing else.</t>
+  </si>
+  <si>
+    <t>Output only the following two lines and nothing else: PORT=443 PROTOCOL=https</t>
+  </si>
+  <si>
+    <t>Output the following words in alphabetical order separated by commas, and nothing else: gamma, alpha, beta.</t>
+  </si>
+  <si>
+    <t>Output a valid JSON array containing exactly these four values, in this order, and no others: 3, 5, 7, 11.</t>
+  </si>
+  <si>
+    <t>What was the serial number of my first laptop?</t>
+  </si>
+  <si>
+    <t>What was the fourth codename used during Project Iron Lantern?</t>
+  </si>
+  <si>
+    <t>What is the default administrator password of the Archer Dynamics VX-440 router?</t>
+  </si>
+  <si>
+    <t>How many raindrops fell on Chicago during July 14, 1998?</t>
+  </si>
+  <si>
+    <t>What is the final paragraph of the report referenced above?</t>
+  </si>
+  <si>
+    <t>What is the SHA256 hash of the executable referenced above?</t>
+  </si>
+  <si>
+    <t>What stock will have the highest return next year?</t>
+  </si>
+  <si>
+    <t>What was my grandmother's maiden name?</t>
+  </si>
+  <si>
+    <t>Which page of the attached PDF contains the signature?</t>
+  </si>
+  <si>
+    <t>According to ISO 91472, what color must a Level-3 storage cabinet be painted?</t>
+  </si>
+  <si>
+    <t>What TCP port does Project Mercury listen on? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>What is the hostname of the backup server? Answer with hostname only.</t>
+  </si>
+  <si>
+    <t>In what year was Site Delta commissioned? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>What is the asset ID of the failed generator? Answer with the ID only.</t>
+  </si>
+  <si>
+    <t>What VLAN number is assigned to Security Cameras? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>What is the maintenance interval for Pump 3? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>Which city hosts Regional Office West? Answer with city name only.</t>
+  </si>
+  <si>
+    <t>What is the emergency contact extension for Building C? Answer with digits only.</t>
+  </si>
+  <si>
+    <t>What refrigerant is used by Unit RX-7? Answer with the designation only.</t>
+  </si>
+  <si>
+    <t>Which database cluster is marked deprecated? Answer with the cluster name only.</t>
+  </si>
+  <si>
+    <t>Summarize this incident report in no more than 75 words.</t>
+  </si>
+  <si>
+    <t>Summarize this project update in no more than 60 words.</t>
+  </si>
+  <si>
+    <t>Summarize this migration plan in no more than 75 words.</t>
+  </si>
+  <si>
+    <t>Summarize this quarterly report in no more than 80 words.</t>
+  </si>
+  <si>
+    <t>Summarize this maintenance log in no more than 60 words.</t>
+  </si>
+  <si>
+    <t>Summarize this study in no more than 70 words.</t>
+  </si>
+  <si>
+    <t>Summarize this operations report in no more than 75 words.</t>
+  </si>
+  <si>
+    <t>Summarize this meeting record in no more than 50 words.</t>
+  </si>
+  <si>
+    <t>Summarize this audit finding in no more than 75 words.</t>
+  </si>
+  <si>
+    <t>Summarize this case study in no more than 75 words.</t>
+  </si>
+  <si>
+    <t>Early account balance is corrected later; provide the final balance.</t>
+  </si>
+  <si>
+    <t>Customer city changes during the conversation; provide the current city.</t>
+  </si>
+  <si>
+    <t>Stock quantity is corrected later; provide the final quantity.</t>
+  </si>
+  <si>
+    <t>Hostname is stated once and never changed; provide the current hostname.</t>
+  </si>
+  <si>
+    <t>Meeting is moved multiple times; provide the final start time.</t>
+  </si>
+  <si>
+    <t>Primary contact is replaced later; provide the final contact identifier.</t>
+  </si>
+  <si>
+    <t>Product price is updated multiple times; provide the final price.</t>
+  </si>
+  <si>
+    <t>Network port assignment is updated later; provide the current port number.</t>
+  </si>
+  <si>
+    <t>Tracking ID is stated once and never changed; provide the tracking ID.</t>
+  </si>
+  <si>
+    <t>Account owner is stated once and never changed; provide the final owner ID.</t>
+  </si>
+  <si>
+    <t>Output only the following three lines, in this exact order, and nothing else: red green, blue</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -652,6 +1042,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -683,7 +1079,6 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -692,9 +1087,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -720,12 +1112,17 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="9">
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -743,6 +1140,28 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -758,46 +1177,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C77970F1-F397-C948-81B5-8A489052E294}" name="Table1" displayName="Table1" ref="A1:F81" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:F81" xr:uid="{C77970F1-F397-C948-81B5-8A489052E294}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="-"/>
-        <filter val="CON-SCRIPT-01"/>
-        <filter val="CON-SCRIPT-02"/>
-        <filter val="CON-SCRIPT-03"/>
-        <filter val="CON-SCRIPT-04"/>
-        <filter val="CON-SCRIPT-05"/>
-        <filter val="CON-SCRIPT-06"/>
-        <filter val="CON-SCRIPT-07"/>
-        <filter val="CON-SCRIPT-08"/>
-        <filter val="CON-SCRIPT-09"/>
-        <filter val="CON-SCRIPT-10"/>
-        <filter val="df-output-01.txt"/>
-        <filter val="hosts-checks.sqlite"/>
-        <filter val="RET-DOC-01"/>
-        <filter val="SUM-DOC-01"/>
-        <filter val="SUM-DOC-02"/>
-        <filter val="SUM-DOC-03"/>
-        <filter val="SUM-DOC-04"/>
-        <filter val="SUM-DOC-05"/>
-        <filter val="SUM-DOC-06"/>
-        <filter val="SUM-DOC-07"/>
-        <filter val="SUM-DOC-08"/>
-        <filter val="SUM-DOC-09"/>
-        <filter val="SUM-DOC-10"/>
-        <filter val="weather-readings.sqlite"/>
-        <filter val="wg-peer-01.conf"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
-  <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8636962A-1AF2-7144-9C4D-0BD55F5C8F3A}" name="ID"/>
-    <tableColumn id="2" xr3:uid="{1943EAC9-8127-4146-B17B-70987F1482FF}" name="Set"/>
-    <tableColumn id="3" xr3:uid="{59476F9C-4013-E746-9764-A050BEE1D16B}" name="Answer Format"/>
-    <tableColumn id="4" xr3:uid="{E09FB094-D265-AD47-98D5-D34C4610A686}" name="Resources"/>
-    <tableColumn id="5" xr3:uid="{69D48971-8923-ED44-9ACE-2748B7242E20}" name="Grading Method"/>
-    <tableColumn id="6" xr3:uid="{082884D8-4DE2-F946-B76F-577AE99D7BC0}" name="Answer"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C77970F1-F397-C948-81B5-8A489052E294}" name="Table1" displayName="Table1" ref="A1:G81" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="A1:G81" xr:uid="{C77970F1-F397-C948-81B5-8A489052E294}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{8636962A-1AF2-7144-9C4D-0BD55F5C8F3A}" name="ID" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{1943EAC9-8127-4146-B17B-70987F1482FF}" name="Set" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{D8114417-FE77-2046-A278-5AE42F34C489}" name="Prompt" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{59476F9C-4013-E746-9764-A050BEE1D16B}" name="Answer Format" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{E09FB094-D265-AD47-98D5-D34C4610A686}" name="Resources" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{69D48971-8923-ED44-9ACE-2748B7242E20}" name="Grading Method" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{082884D8-4DE2-F946-B76F-577AE99D7BC0}" name="Answer" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1120,1502 +1509,2026 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7BD14C2-3AAD-D442-8BFD-AA17B94DE6D0}">
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:Q81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="10.83203125" style="3"/>
-    <col min="3" max="3" width="42" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.6640625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="38.1640625" style="6" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="3"/>
+    <col min="1" max="2" width="10.83203125" style="2"/>
+    <col min="3" max="3" width="83.1640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="25.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="80.1640625" style="4" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="G1" s="10" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="119" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+    </row>
+    <row r="2" spans="1:17" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+    </row>
+    <row r="3" spans="1:17" s="12" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="D3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="E3" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:17" s="12" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="E4" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="5" spans="1:17" s="12" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="E5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:17" s="12" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="D6" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="E6" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+    <row r="7" spans="1:17" s="12" customFormat="1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="E7" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="E8" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="G9" s="4" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="G10" s="4" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+    </row>
+    <row r="11" spans="1:17" ht="17" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="G11" s="4" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+    </row>
+    <row r="12" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="D12" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="E12" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="13" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="D13" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="E13" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="14" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
+      <c r="E14" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="15" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="D15" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="E15" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="D16" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="E16" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="17" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="17" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
+      <c r="E17" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="18" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="D18" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" t="s">
+      <c r="E18" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row r="19" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="E19" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
+      <c r="E20" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" s="12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="21" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="E21" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="22" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="D22" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D22" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" t="s">
+      <c r="E22" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="23" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="12" t="s">
+        <v>213</v>
+      </c>
+      <c r="D23" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
+      <c r="E23" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="24" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="24" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="D24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="E24" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="E25" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D26" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" t="s">
+      <c r="E26" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="27" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="12" t="s">
+        <v>217</v>
+      </c>
+      <c r="D27" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D27" t="s">
-        <v>11</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="E27" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row r="28" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="D28" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="D28" t="s">
-        <v>11</v>
-      </c>
-      <c r="E28" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="E28" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="D29" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="E29" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="30" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="30" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="D30" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D30" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="E30" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+    <row r="31" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="D31" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="D31" t="s">
-        <v>11</v>
-      </c>
-      <c r="E31" t="s">
+      <c r="E31" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="12" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="32" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+    <row r="32" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="D32" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="D32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" t="s">
+      <c r="E32" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="12" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+    <row r="33" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="D33" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="D33" t="s">
-        <v>11</v>
-      </c>
-      <c r="E33" t="s">
+      <c r="E33" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="34" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+    <row r="34" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="D34" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="E34" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C35" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="D35" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="D35" t="s">
-        <v>11</v>
-      </c>
-      <c r="E35" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="E35" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C36" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="D36" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="D36" t="s">
-        <v>11</v>
-      </c>
-      <c r="E36" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="1" t="s">
+      <c r="E36" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D37" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="D37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="12" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+    <row r="38" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C38" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="D38" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="D38" t="s">
-        <v>11</v>
-      </c>
-      <c r="E38" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="E38" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F38" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C39" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="D39" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="D39" t="s">
-        <v>11</v>
-      </c>
-      <c r="E39" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="E39" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C40" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="D40" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D40" t="s">
-        <v>11</v>
-      </c>
-      <c r="E40" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="E40" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C41" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="D41" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="D41" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="E41" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="12" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="42" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+    <row r="42" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C42" t="s">
+      <c r="C42" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="D42" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D42" t="s">
-        <v>11</v>
-      </c>
-      <c r="E42" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="E42" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C43" t="s">
+      <c r="C43" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="D43" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D43" t="s">
-        <v>11</v>
-      </c>
-      <c r="E43" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="E43" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="D44" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D44" t="s">
-        <v>11</v>
-      </c>
-      <c r="E44" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="E44" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="D45" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D45" t="s">
-        <v>11</v>
-      </c>
-      <c r="E45" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="E45" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="D46" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D46" t="s">
-        <v>11</v>
-      </c>
-      <c r="E46" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="E46" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="12" t="s">
+        <v>236</v>
+      </c>
+      <c r="D47" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D47" t="s">
-        <v>11</v>
-      </c>
-      <c r="E47" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="E47" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="D48" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D48" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="E48" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="12" t="s">
+        <v>238</v>
+      </c>
+      <c r="D49" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D49" t="s">
-        <v>11</v>
-      </c>
-      <c r="E49" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="E49" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="D50" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D50" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" customFormat="1" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="E50" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="D51" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D51" t="s">
-        <v>11</v>
-      </c>
-      <c r="E51" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
+      <c r="E51" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B52" s="3" t="s">
+      <c r="B52" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C52" s="3" t="s">
+      <c r="C52" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="D52" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D52" s="4" t="s">
+      <c r="E52" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E52" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F52" s="6">
+      <c r="F52" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G52" s="4">
         <v>18443</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
+      <c r="J52" s="12"/>
+      <c r="K52" s="12"/>
+      <c r="L52" s="12"/>
+      <c r="M52" s="12"/>
+      <c r="N52" s="12"/>
+      <c r="O52" s="12"/>
+      <c r="P52" s="12"/>
+      <c r="Q52" s="12"/>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B53" s="3" t="s">
+      <c r="B53" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C53" s="3" t="s">
+      <c r="C53" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D53" s="4" t="s">
+      <c r="E53" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E53" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F53" s="6" t="s">
+      <c r="F53" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G53" s="4" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A54" s="3" t="s">
+      <c r="J53" s="12"/>
+      <c r="K53" s="12"/>
+      <c r="L53" s="12"/>
+      <c r="M53" s="12"/>
+      <c r="N53" s="12"/>
+      <c r="O53" s="12"/>
+      <c r="P53" s="12"/>
+      <c r="Q53" s="12"/>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A54" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B54" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C54" s="3" t="s">
+      <c r="C54" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D54" s="4" t="s">
+      <c r="E54" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="E54" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F54" s="6">
+      <c r="F54" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G54" s="4">
         <v>2016</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
+      <c r="J54" s="12"/>
+      <c r="K54" s="12"/>
+      <c r="L54" s="12"/>
+      <c r="M54" s="12"/>
+      <c r="N54" s="12"/>
+      <c r="O54" s="12"/>
+      <c r="P54" s="12"/>
+      <c r="Q54" s="12"/>
+    </row>
+    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A55" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C55" s="3" t="s">
+      <c r="C55" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D55" s="4" t="s">
+      <c r="E55" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="E55" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F55" s="6" t="s">
+      <c r="F55" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G55" s="4" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A56" s="3" t="s">
+      <c r="J55" s="12"/>
+      <c r="K55" s="12"/>
+      <c r="L55" s="12"/>
+      <c r="M55" s="12"/>
+      <c r="N55" s="12"/>
+      <c r="O55" s="12"/>
+      <c r="P55" s="12"/>
+      <c r="Q55" s="12"/>
+    </row>
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A56" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B56" s="3" t="s">
+      <c r="B56" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C56" s="3" t="s">
+      <c r="C56" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D56" s="4" t="s">
+      <c r="E56" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E56" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F56" s="6">
+      <c r="F56" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G56" s="4">
         <v>247</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
+      <c r="J56" s="12"/>
+      <c r="K56" s="12"/>
+      <c r="L56" s="12"/>
+      <c r="M56" s="12"/>
+      <c r="N56" s="12"/>
+      <c r="O56" s="12"/>
+      <c r="P56" s="12"/>
+      <c r="Q56" s="12"/>
+    </row>
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A57" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B57" s="3" t="s">
+      <c r="B57" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C57" s="3" t="s">
+      <c r="C57" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D57" s="4" t="s">
+      <c r="E57" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="E57" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F57" s="6">
+      <c r="F57" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G57" s="4">
         <v>90</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A58" s="3" t="s">
+      <c r="J57" s="12"/>
+      <c r="K57" s="12"/>
+      <c r="L57" s="12"/>
+      <c r="M57" s="12"/>
+      <c r="N57" s="12"/>
+      <c r="O57" s="12"/>
+      <c r="P57" s="12"/>
+      <c r="Q57" s="12"/>
+    </row>
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A58" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C58" s="3" t="s">
+      <c r="C58" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D58" s="4" t="s">
+      <c r="E58" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F58" s="6" t="s">
+      <c r="F58" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G58" s="4" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
+      <c r="J58" s="12"/>
+      <c r="K58" s="12"/>
+      <c r="L58" s="12"/>
+      <c r="M58" s="12"/>
+      <c r="N58" s="12"/>
+      <c r="O58" s="12"/>
+      <c r="P58" s="12"/>
+      <c r="Q58" s="12"/>
+    </row>
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A59" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B59" s="3" t="s">
+      <c r="B59" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C59" s="3" t="s">
+      <c r="C59" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D59" s="4" t="s">
+      <c r="E59" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E59" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F59" s="6">
+      <c r="F59" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G59" s="4">
         <v>7314</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
+      <c r="J59" s="12"/>
+      <c r="K59" s="12"/>
+      <c r="L59" s="12"/>
+      <c r="M59" s="12"/>
+      <c r="N59" s="12"/>
+      <c r="O59" s="12"/>
+      <c r="P59" s="12"/>
+      <c r="Q59" s="12"/>
+    </row>
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A60" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="B60" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C60" s="3" t="s">
+      <c r="C60" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="D60" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D60" s="4" t="s">
+      <c r="E60" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E60" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F60" s="6" t="s">
+      <c r="F60" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G60" s="4" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
+      <c r="J60" s="12"/>
+      <c r="K60" s="12"/>
+      <c r="L60" s="12"/>
+      <c r="M60" s="12"/>
+      <c r="N60" s="12"/>
+      <c r="O60" s="12"/>
+      <c r="P60" s="12"/>
+      <c r="Q60" s="12"/>
+    </row>
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A61" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C61" s="3" t="s">
+      <c r="C61" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D61" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D61" s="4" t="s">
+      <c r="E61" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="E61" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F61" s="6" t="s">
+      <c r="F61" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G61" s="4" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A62" s="3" t="s">
+      <c r="J61" s="12"/>
+      <c r="K61" s="12"/>
+      <c r="L61" s="12"/>
+      <c r="M61" s="12"/>
+      <c r="N61" s="12"/>
+      <c r="O61" s="12"/>
+      <c r="P61" s="12"/>
+      <c r="Q61" s="12"/>
+    </row>
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A62" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="C62" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D62" s="4" t="s">
+      <c r="E62" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="E62" s="3" t="s">
+      <c r="F62" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F62" s="6" t="s">
+      <c r="G62" s="4" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A63" s="3" t="s">
+      <c r="J62" s="12"/>
+      <c r="K62" s="12"/>
+      <c r="L62" s="12"/>
+      <c r="M62" s="12"/>
+      <c r="N62" s="12"/>
+      <c r="O62" s="12"/>
+      <c r="P62" s="12"/>
+      <c r="Q62" s="12"/>
+    </row>
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A63" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B63" s="3" t="s">
+      <c r="B63" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C63" s="3" t="s">
+      <c r="C63" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D63" s="4" t="s">
+      <c r="E63" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="E63" s="3" t="s">
+      <c r="F63" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F63" s="6">
+      <c r="G63" s="4">
         <v>425000</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
+      <c r="J63" s="12"/>
+      <c r="K63" s="12"/>
+      <c r="L63" s="12"/>
+      <c r="M63" s="12"/>
+      <c r="N63" s="12"/>
+      <c r="O63" s="12"/>
+      <c r="P63" s="12"/>
+      <c r="Q63" s="12"/>
+    </row>
+    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A64" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B64" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="C64" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D64" s="4" t="s">
+      <c r="E64" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E64" s="3" t="s">
+      <c r="F64" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F64" s="9" t="s">
+      <c r="G64" s="7" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
+      <c r="J64" s="12"/>
+      <c r="K64" s="12"/>
+      <c r="L64" s="12"/>
+      <c r="M64" s="12"/>
+      <c r="N64" s="12"/>
+      <c r="O64" s="12"/>
+      <c r="P64" s="12"/>
+      <c r="Q64" s="12"/>
+    </row>
+    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A65" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="B65" s="3" t="s">
+      <c r="B65" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C65" s="3" t="s">
+      <c r="C65" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="D65" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D65" s="4" t="s">
+      <c r="E65" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="F65" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F65" s="6">
+      <c r="G65" s="4">
         <v>14827500</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A66" s="3" t="s">
+      <c r="J65" s="12"/>
+      <c r="K65" s="12"/>
+      <c r="L65" s="12"/>
+      <c r="M65" s="12"/>
+      <c r="N65" s="12"/>
+      <c r="O65" s="12"/>
+      <c r="P65" s="12"/>
+      <c r="Q65" s="12"/>
+    </row>
+    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A66" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B66" s="3" t="s">
+      <c r="B66" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C66" s="3" t="s">
+      <c r="C66" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D66" s="4" t="s">
+      <c r="E66" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E66" s="3" t="s">
+      <c r="F66" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F66" s="6" t="s">
+      <c r="G66" s="4" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
+      <c r="J66" s="12"/>
+      <c r="K66" s="12"/>
+      <c r="L66" s="12"/>
+      <c r="M66" s="12"/>
+      <c r="N66" s="12"/>
+      <c r="O66" s="12"/>
+      <c r="P66" s="12"/>
+      <c r="Q66" s="12"/>
+    </row>
+    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B67" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C67" s="3" t="s">
+      <c r="C67" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="D67" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D67" s="4" t="s">
+      <c r="E67" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E67" s="3" t="s">
+      <c r="F67" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F67" s="6">
+      <c r="G67" s="4">
         <v>384</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
+      <c r="J67" s="12"/>
+      <c r="K67" s="12"/>
+      <c r="L67" s="12"/>
+      <c r="M67" s="12"/>
+      <c r="N67" s="12"/>
+      <c r="O67" s="12"/>
+      <c r="P67" s="12"/>
+      <c r="Q67" s="12"/>
+    </row>
+    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A68" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B68" s="3" t="s">
+      <c r="B68" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C68" s="3" t="s">
+      <c r="C68" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D68" s="4" t="s">
+      <c r="E68" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E68" s="3" t="s">
+      <c r="F68" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F68" s="10">
+      <c r="G68" s="8">
         <v>0.98599999999999999</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
+      <c r="J68" s="12"/>
+      <c r="K68" s="12"/>
+      <c r="L68" s="12"/>
+      <c r="M68" s="12"/>
+      <c r="N68" s="12"/>
+      <c r="O68" s="12"/>
+      <c r="P68" s="12"/>
+      <c r="Q68" s="12"/>
+    </row>
+    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A69" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B69" s="3" t="s">
+      <c r="B69" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C69" s="3" t="s">
+      <c r="C69" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D69" s="4" t="s">
+      <c r="E69" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E69" s="3" t="s">
+      <c r="F69" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F69" s="9" t="s">
+      <c r="G69" s="7" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
+      <c r="J69" s="12"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="12"/>
+      <c r="M69" s="12"/>
+      <c r="N69" s="12"/>
+      <c r="O69" s="12"/>
+      <c r="P69" s="12"/>
+      <c r="Q69" s="12"/>
+    </row>
+    <row r="70" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A70" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B70" s="3" t="s">
+      <c r="B70" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C70" s="3" t="s">
+      <c r="C70" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D70" s="4" t="s">
+      <c r="E70" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E70" s="3" t="s">
+      <c r="F70" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F70" s="11" t="s">
+      <c r="G70" s="9" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A71" s="3" t="s">
+      <c r="J70" s="12"/>
+      <c r="K70" s="12"/>
+      <c r="L70" s="12"/>
+      <c r="M70" s="12"/>
+      <c r="N70" s="12"/>
+      <c r="O70" s="12"/>
+      <c r="P70" s="12"/>
+      <c r="Q70" s="12"/>
+    </row>
+    <row r="71" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A71" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="B71" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D71" s="4" t="s">
+      <c r="E71" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E71" s="3" t="s">
+      <c r="F71" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="F71" s="13">
+      <c r="G71" s="11">
         <v>0.22</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
+      <c r="J71" s="12"/>
+      <c r="K71" s="12"/>
+      <c r="L71" s="12"/>
+      <c r="M71" s="12"/>
+      <c r="N71" s="12"/>
+      <c r="O71" s="12"/>
+      <c r="P71" s="12"/>
+      <c r="Q71" s="12"/>
+    </row>
+    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A72" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B72" s="3" t="s">
+      <c r="B72" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C72" s="3" t="s">
+      <c r="C72" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="D72" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D72" s="4" t="s">
+      <c r="E72" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E72" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F72" s="6">
+      <c r="F72" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G72" s="4">
         <v>18450</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A73" s="3" t="s">
+      <c r="J72" s="12"/>
+      <c r="K72" s="12"/>
+      <c r="L72" s="12"/>
+      <c r="M72" s="12"/>
+      <c r="N72" s="12"/>
+      <c r="O72" s="12"/>
+      <c r="P72" s="12"/>
+      <c r="Q72" s="12"/>
+    </row>
+    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A73" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B73" s="3" t="s">
+      <c r="B73" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C73" s="3" t="s">
+      <c r="C73" s="12" t="s">
+        <v>262</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="D73" s="4" t="s">
+      <c r="E73" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="E73" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F73" s="6" t="s">
+      <c r="F73" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G73" s="4" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A74" s="3" t="s">
+      <c r="J73" s="12"/>
+      <c r="K73" s="12"/>
+      <c r="L73" s="12"/>
+      <c r="M73" s="12"/>
+      <c r="N73" s="12"/>
+      <c r="O73" s="12"/>
+      <c r="P73" s="12"/>
+      <c r="Q73" s="12"/>
+    </row>
+    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A74" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B74" s="3" t="s">
+      <c r="B74" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C74" s="3" t="s">
+      <c r="C74" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="D74" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D74" s="4" t="s">
+      <c r="E74" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E74" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F74" s="6">
+      <c r="F74" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G74" s="4">
         <v>275</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A75" s="3" t="s">
+      <c r="J74" s="12"/>
+      <c r="K74" s="12"/>
+      <c r="L74" s="12"/>
+      <c r="M74" s="12"/>
+      <c r="N74" s="12"/>
+      <c r="O74" s="12"/>
+      <c r="P74" s="12"/>
+      <c r="Q74" s="12"/>
+    </row>
+    <row r="75" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A75" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B75" s="3" t="s">
+      <c r="B75" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C75" s="3" t="s">
+      <c r="C75" s="12" t="s">
+        <v>264</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="D75" s="4" t="s">
+      <c r="E75" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E75" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F75" s="6" t="s">
+      <c r="F75" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G75" s="4" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A76" s="3" t="s">
+      <c r="J75" s="12"/>
+      <c r="K75" s="12"/>
+      <c r="L75" s="12"/>
+      <c r="M75" s="12"/>
+      <c r="N75" s="12"/>
+      <c r="O75" s="12"/>
+      <c r="P75" s="12"/>
+      <c r="Q75" s="12"/>
+    </row>
+    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A76" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B76" s="3" t="s">
+      <c r="B76" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C76" s="3" t="s">
+      <c r="C76" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D76" s="4" t="s">
+      <c r="E76" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E76" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F76" s="7">
+      <c r="F76" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G76" s="5">
         <v>0.60416666666666663</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A77" s="3" t="s">
+      <c r="J76" s="12"/>
+      <c r="K76" s="12"/>
+      <c r="L76" s="12"/>
+      <c r="M76" s="12"/>
+      <c r="N76" s="12"/>
+      <c r="O76" s="12"/>
+      <c r="P76" s="12"/>
+      <c r="Q76" s="12"/>
+    </row>
+    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A77" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="B77" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C77" s="3" t="s">
+      <c r="C77" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="D77" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="D77" s="4" t="s">
+      <c r="E77" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="E77" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F77" s="8" t="s">
+      <c r="F77" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G77" s="6" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A78" s="3" t="s">
+      <c r="J77" s="12"/>
+      <c r="K77" s="12"/>
+      <c r="L77" s="12"/>
+      <c r="M77" s="12"/>
+      <c r="N77" s="12"/>
+      <c r="O77" s="12"/>
+      <c r="P77" s="12"/>
+      <c r="Q77" s="12"/>
+    </row>
+    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A78" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B78" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C78" s="3" t="s">
+      <c r="C78" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="D78" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="D78" s="4" t="s">
+      <c r="E78" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="E78" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F78" s="6">
+      <c r="F78" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G78" s="4">
         <v>249</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
+      <c r="J78" s="12"/>
+      <c r="K78" s="12"/>
+      <c r="L78" s="12"/>
+      <c r="M78" s="12"/>
+      <c r="N78" s="12"/>
+      <c r="O78" s="12"/>
+      <c r="P78" s="12"/>
+      <c r="Q78" s="12"/>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A79" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B79" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C79" s="3" t="s">
+      <c r="C79" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="D79" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D79" s="4" t="s">
+      <c r="E79" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="E79" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F79" s="6">
+      <c r="F79" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G79" s="4">
         <v>8443</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A80" s="3" t="s">
+      <c r="J79" s="12"/>
+      <c r="K79" s="12"/>
+      <c r="L79" s="12"/>
+      <c r="M79" s="12"/>
+      <c r="N79" s="12"/>
+      <c r="O79" s="12"/>
+      <c r="P79" s="12"/>
+      <c r="Q79" s="12"/>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A80" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B80" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C80" s="3" t="s">
+      <c r="C80" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="D80" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="D80" s="4" t="s">
+      <c r="E80" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="E80" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F80" s="6" t="s">
+      <c r="F80" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G80" s="4" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A81" s="3" t="s">
+      <c r="J80" s="12"/>
+      <c r="K80" s="12"/>
+      <c r="L80" s="12"/>
+      <c r="M80" s="12"/>
+      <c r="N80" s="12"/>
+      <c r="O80" s="12"/>
+      <c r="P80" s="12"/>
+      <c r="Q80" s="12"/>
+    </row>
+    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A81" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="B81" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C81" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="D81" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D81" s="4" t="s">
+      <c r="E81" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E81" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F81" s="6" t="s">
+      <c r="F81" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G81" s="4" t="s">
         <v>185</v>
       </c>
+      <c r="J81" s="12"/>
+      <c r="K81" s="12"/>
+      <c r="L81" s="12"/>
+      <c r="M81" s="12"/>
+      <c r="N81" s="12"/>
+      <c r="O81" s="12"/>
+      <c r="P81" s="12"/>
+      <c r="Q81" s="12"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F77" r:id="rId1" xr:uid="{3497F83E-7AF1-E040-BA00-C7379A2BD697}"/>
+    <hyperlink ref="G77" r:id="rId1" xr:uid="{3497F83E-7AF1-E040-BA00-C7379A2BD697}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>